<commit_message>
update Genesee county foc address
</commit_message>
<xml_diff>
--- a/docassemble/mlhframework/data/sources/michigan_court_info.xlsx
+++ b/docassemble/mlhframework/data/sources/michigan_court_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://miadvocacyprog-my.sharepoint.com/personal/ekressmiller_lsscm_org/Documents/Attachments/Desktop/Active Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EmilyKressMiller\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6210CF26-958D-43DC-BF4F-D246EE51CB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52364585-4DC9-4306-95DE-08E1F29F7797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Courts" sheetId="1" r:id="rId1"/>
@@ -230,7 +230,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3603" uniqueCount="1697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3603" uniqueCount="1696">
   <si>
     <t>address_county</t>
   </si>
@@ -4276,12 +4276,6 @@
     <t>7th Circuit Court - Genesee Co. FOC</t>
   </si>
   <si>
-    <t>1101 Beach St.</t>
-  </si>
-  <si>
-    <t>Genesee Co. Administration Bldg.</t>
-  </si>
-  <si>
     <t>(810) 257-3300</t>
   </si>
   <si>
@@ -5321,6 +5315,9 @@
   </si>
   <si>
     <t>(231) 779-9510</t>
+  </si>
+  <si>
+    <t>Suite 2500</t>
   </si>
 </sst>
 </file>
@@ -15696,16 +15693,17 @@
         <v>1347</v>
       </c>
       <c r="F266" s="3" t="s">
-        <v>1348</v>
+        <v>681</v>
+      </c>
+      <c r="G266" s="3" t="s">
+        <v>1695</v>
       </c>
       <c r="H266" s="5" t="s">
         <v>682</v>
       </c>
-      <c r="I266" s="3" t="s">
-        <v>1349</v>
-      </c>
+      <c r="I266" s="3"/>
       <c r="J266" s="3" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="L266" s="3" t="str">
         <f t="shared" si="3"/>
@@ -15730,7 +15728,7 @@
         <v>138</v>
       </c>
       <c r="E267" s="3" t="s">
-        <v>1351</v>
+        <v>1349</v>
       </c>
       <c r="F267" s="3" t="s">
         <v>196</v>
@@ -15767,7 +15765,7 @@
         <v>200</v>
       </c>
       <c r="E268" s="3" t="s">
-        <v>1352</v>
+        <v>1350</v>
       </c>
       <c r="F268" s="3" t="s">
         <v>202</v>
@@ -15804,7 +15802,7 @@
         <v>49</v>
       </c>
       <c r="E269" s="3" t="s">
-        <v>1353</v>
+        <v>1351</v>
       </c>
       <c r="F269" s="3" t="s">
         <v>208</v>
@@ -15841,7 +15839,7 @@
         <v>145</v>
       </c>
       <c r="E270" s="3" t="s">
-        <v>1354</v>
+        <v>1352</v>
       </c>
       <c r="F270" s="3" t="s">
         <v>213</v>
@@ -15853,7 +15851,7 @@
         <v>73</v>
       </c>
       <c r="J270" s="3" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="L270" s="3" t="str">
         <f t="shared" si="3"/>
@@ -15878,16 +15876,16 @@
         <v>219</v>
       </c>
       <c r="E271" s="3" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="F271" s="3" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
       <c r="H271" s="5" t="s">
         <v>739</v>
       </c>
       <c r="J271" s="3" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
       <c r="L271" s="3" t="str">
         <f t="shared" si="3"/>
@@ -15912,7 +15910,7 @@
         <v>62</v>
       </c>
       <c r="E272" s="3" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="F272" s="5" t="s">
         <v>225</v>
@@ -15949,7 +15947,7 @@
         <v>230</v>
       </c>
       <c r="E273" s="3" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
       <c r="F273" s="5" t="s">
         <v>232</v>
@@ -15986,16 +15984,16 @@
         <v>237</v>
       </c>
       <c r="E274" s="3" t="s">
+        <v>1359</v>
+      </c>
+      <c r="F274" s="3" t="s">
+        <v>1360</v>
+      </c>
+      <c r="H274" s="5" t="s">
         <v>1361</v>
       </c>
-      <c r="F274" s="3" t="s">
+      <c r="J274" s="3" t="s">
         <v>1362</v>
-      </c>
-      <c r="H274" s="5" t="s">
-        <v>1363</v>
-      </c>
-      <c r="J274" s="3" t="s">
-        <v>1364</v>
       </c>
       <c r="L274" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16020,16 +16018,16 @@
         <v>245</v>
       </c>
       <c r="E275" s="3" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="F275" s="3" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="H275" s="5" t="s">
         <v>769</v>
       </c>
       <c r="J275" s="3" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="L275" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16054,16 +16052,16 @@
         <v>21</v>
       </c>
       <c r="E276" s="3" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="F276" s="3" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
       <c r="H276" s="5" t="s">
         <v>772</v>
       </c>
       <c r="J276" s="3" t="s">
-        <v>1370</v>
+        <v>1368</v>
       </c>
       <c r="L276" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16088,13 +16086,13 @@
         <v>167</v>
       </c>
       <c r="E277" s="3" t="s">
-        <v>1371</v>
+        <v>1369</v>
       </c>
       <c r="F277" s="3" t="s">
         <v>259</v>
       </c>
       <c r="G277" s="3" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
       <c r="H277" s="5" t="s">
         <v>775</v>
@@ -16103,7 +16101,7 @@
         <v>261</v>
       </c>
       <c r="J277" s="3" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="L277" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16128,7 +16126,7 @@
         <v>264</v>
       </c>
       <c r="E278" s="3" t="s">
-        <v>1374</v>
+        <v>1372</v>
       </c>
       <c r="F278" s="3" t="s">
         <v>266</v>
@@ -16165,16 +16163,16 @@
         <v>271</v>
       </c>
       <c r="E279" s="3" t="s">
+        <v>1373</v>
+      </c>
+      <c r="F279" s="3" t="s">
+        <v>1374</v>
+      </c>
+      <c r="H279" s="5" t="s">
         <v>1375</v>
       </c>
-      <c r="F279" s="3" t="s">
+      <c r="J279" s="3" t="s">
         <v>1376</v>
-      </c>
-      <c r="H279" s="5" t="s">
-        <v>1377</v>
-      </c>
-      <c r="J279" s="3" t="s">
-        <v>1378</v>
       </c>
       <c r="L279" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16199,16 +16197,16 @@
         <v>278</v>
       </c>
       <c r="E280" s="3" t="s">
+        <v>1377</v>
+      </c>
+      <c r="F280" s="3" t="s">
+        <v>1378</v>
+      </c>
+      <c r="H280" s="5" t="s">
         <v>1379</v>
       </c>
-      <c r="F280" s="3" t="s">
+      <c r="J280" s="3" t="s">
         <v>1380</v>
-      </c>
-      <c r="H280" s="5" t="s">
-        <v>1381</v>
-      </c>
-      <c r="J280" s="3" t="s">
-        <v>1382</v>
       </c>
       <c r="L280" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16233,7 +16231,7 @@
         <v>153</v>
       </c>
       <c r="E281" s="3" t="s">
-        <v>1383</v>
+        <v>1381</v>
       </c>
       <c r="F281" s="3" t="s">
         <v>285</v>
@@ -16245,7 +16243,7 @@
         <v>288</v>
       </c>
       <c r="J281" s="3" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="L281" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16270,16 +16268,16 @@
         <v>291</v>
       </c>
       <c r="E282" s="3" t="s">
+        <v>1383</v>
+      </c>
+      <c r="F282" s="3" t="s">
+        <v>1384</v>
+      </c>
+      <c r="H282" s="5" t="s">
         <v>1385</v>
       </c>
-      <c r="F282" s="3" t="s">
+      <c r="J282" s="3" t="s">
         <v>1386</v>
-      </c>
-      <c r="H282" s="5" t="s">
-        <v>1387</v>
-      </c>
-      <c r="J282" s="3" t="s">
-        <v>1388</v>
       </c>
       <c r="L282" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16304,7 +16302,7 @@
         <v>62</v>
       </c>
       <c r="E283" s="3" t="s">
-        <v>1389</v>
+        <v>1387</v>
       </c>
       <c r="F283" s="3" t="s">
         <v>298</v>
@@ -16341,7 +16339,7 @@
         <v>303</v>
       </c>
       <c r="E284" s="3" t="s">
-        <v>1390</v>
+        <v>1388</v>
       </c>
       <c r="F284" s="3" t="s">
         <v>305</v>
@@ -16350,7 +16348,7 @@
         <v>831</v>
       </c>
       <c r="J284" s="3" t="s">
-        <v>1391</v>
+        <v>1389</v>
       </c>
       <c r="L284" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16375,7 +16373,7 @@
         <v>310</v>
       </c>
       <c r="E285" s="3" t="s">
-        <v>1392</v>
+        <v>1390</v>
       </c>
       <c r="F285" s="3" t="s">
         <v>312</v>
@@ -16387,7 +16385,7 @@
         <v>314</v>
       </c>
       <c r="J285" s="3" t="s">
-        <v>1393</v>
+        <v>1391</v>
       </c>
       <c r="L285" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16412,7 +16410,7 @@
         <v>49</v>
       </c>
       <c r="E286" s="3" t="s">
-        <v>1394</v>
+        <v>1392</v>
       </c>
       <c r="F286" s="3" t="s">
         <v>317</v>
@@ -16446,7 +16444,7 @@
         <v>322</v>
       </c>
       <c r="E287" s="3" t="s">
-        <v>1395</v>
+        <v>1393</v>
       </c>
       <c r="F287" s="3" t="s">
         <v>324</v>
@@ -16483,7 +16481,7 @@
         <v>329</v>
       </c>
       <c r="E288" s="3" t="s">
-        <v>1396</v>
+        <v>1394</v>
       </c>
       <c r="F288" s="3" t="s">
         <v>331</v>
@@ -16492,7 +16490,7 @@
         <v>843</v>
       </c>
       <c r="J288" s="3" t="s">
-        <v>1397</v>
+        <v>1395</v>
       </c>
       <c r="L288" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16517,7 +16515,7 @@
         <v>29</v>
       </c>
       <c r="E289" s="3" t="s">
-        <v>1398</v>
+        <v>1396</v>
       </c>
       <c r="F289" s="3" t="s">
         <v>336</v>
@@ -16554,7 +16552,7 @@
         <v>29</v>
       </c>
       <c r="E290" s="3" t="s">
-        <v>1399</v>
+        <v>1397</v>
       </c>
       <c r="F290" s="3" t="s">
         <v>341</v>
@@ -16591,19 +16589,19 @@
         <v>346</v>
       </c>
       <c r="E291" s="3" t="s">
-        <v>1400</v>
+        <v>1398</v>
       </c>
       <c r="F291" s="3" t="s">
         <v>348</v>
       </c>
       <c r="H291" s="5" t="s">
-        <v>1401</v>
+        <v>1399</v>
       </c>
       <c r="I291" s="3" t="s">
         <v>350</v>
       </c>
       <c r="J291" s="3" t="s">
-        <v>1402</v>
+        <v>1400</v>
       </c>
       <c r="L291" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16628,7 +16626,7 @@
         <v>82</v>
       </c>
       <c r="E292" s="3" t="s">
-        <v>1403</v>
+        <v>1401</v>
       </c>
       <c r="F292" s="3" t="s">
         <v>353</v>
@@ -16662,10 +16660,10 @@
         <v>358</v>
       </c>
       <c r="E293" s="3" t="s">
-        <v>1404</v>
+        <v>1402</v>
       </c>
       <c r="F293" s="3" t="s">
-        <v>1405</v>
+        <v>1403</v>
       </c>
       <c r="H293" s="5" t="s">
         <v>923</v>
@@ -16699,7 +16697,7 @@
         <v>365</v>
       </c>
       <c r="E294" s="3" t="s">
-        <v>1406</v>
+        <v>1404</v>
       </c>
       <c r="F294" s="3" t="s">
         <v>367</v>
@@ -16736,7 +16734,7 @@
         <v>372</v>
       </c>
       <c r="E295" s="3" t="s">
-        <v>1407</v>
+        <v>1405</v>
       </c>
       <c r="F295" s="3" t="s">
         <v>374</v>
@@ -16748,7 +16746,7 @@
         <v>376</v>
       </c>
       <c r="J295" s="3" t="s">
-        <v>1408</v>
+        <v>1406</v>
       </c>
       <c r="L295" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16773,10 +16771,10 @@
         <v>167</v>
       </c>
       <c r="E296" s="3" t="s">
-        <v>1409</v>
+        <v>1407</v>
       </c>
       <c r="F296" s="3" t="s">
-        <v>1410</v>
+        <v>1408</v>
       </c>
       <c r="H296" s="5" t="s">
         <v>936</v>
@@ -16785,7 +16783,7 @@
         <v>73</v>
       </c>
       <c r="J296" s="3" t="s">
-        <v>1411</v>
+        <v>1409</v>
       </c>
       <c r="L296" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16810,19 +16808,19 @@
         <v>384</v>
       </c>
       <c r="E297" s="3" t="s">
-        <v>1412</v>
+        <v>1410</v>
       </c>
       <c r="F297" s="3" t="s">
-        <v>1413</v>
+        <v>1411</v>
       </c>
       <c r="H297" s="5" t="s">
         <v>940</v>
       </c>
       <c r="I297" s="3" t="s">
-        <v>1414</v>
+        <v>1412</v>
       </c>
       <c r="J297" s="3" t="s">
-        <v>1415</v>
+        <v>1413</v>
       </c>
       <c r="L297" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16847,7 +16845,7 @@
         <v>391</v>
       </c>
       <c r="E298" s="3" t="s">
-        <v>1416</v>
+        <v>1414</v>
       </c>
       <c r="F298" s="3" t="s">
         <v>393</v>
@@ -16884,7 +16882,7 @@
         <v>399</v>
       </c>
       <c r="E299" s="3" t="s">
-        <v>1417</v>
+        <v>1415</v>
       </c>
       <c r="F299" s="3" t="s">
         <v>401</v>
@@ -16893,7 +16891,7 @@
         <v>954</v>
       </c>
       <c r="J299" s="3" t="s">
-        <v>1418</v>
+        <v>1416</v>
       </c>
       <c r="L299" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16918,10 +16916,10 @@
         <v>245</v>
       </c>
       <c r="E300" s="3" t="s">
-        <v>1419</v>
+        <v>1417</v>
       </c>
       <c r="F300" s="3" t="s">
-        <v>1420</v>
+        <v>1418</v>
       </c>
       <c r="H300" s="5" t="s">
         <v>959</v>
@@ -16930,7 +16928,7 @@
         <v>409</v>
       </c>
       <c r="J300" s="3" t="s">
-        <v>1421</v>
+        <v>1419</v>
       </c>
       <c r="L300" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16955,10 +16953,10 @@
         <v>42</v>
       </c>
       <c r="E301" s="3" t="s">
-        <v>1422</v>
+        <v>1420</v>
       </c>
       <c r="F301" s="3" t="s">
-        <v>1423</v>
+        <v>1421</v>
       </c>
       <c r="H301" s="5" t="s">
         <v>962</v>
@@ -16967,7 +16965,7 @@
         <v>73</v>
       </c>
       <c r="J301" s="3" t="s">
-        <v>1424</v>
+        <v>1422</v>
       </c>
       <c r="L301" s="3" t="str">
         <f t="shared" si="3"/>
@@ -16992,7 +16990,7 @@
         <v>418</v>
       </c>
       <c r="E302" s="3" t="s">
-        <v>1425</v>
+        <v>1423</v>
       </c>
       <c r="F302" s="3" t="s">
         <v>420</v>
@@ -17001,7 +16999,7 @@
         <v>967</v>
       </c>
       <c r="J302" s="3" t="s">
-        <v>1426</v>
+        <v>1424</v>
       </c>
       <c r="L302" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17026,10 +17024,10 @@
         <v>303</v>
       </c>
       <c r="E303" s="3" t="s">
-        <v>1427</v>
+        <v>1425</v>
       </c>
       <c r="F303" s="3" t="s">
-        <v>1428</v>
+        <v>1426</v>
       </c>
       <c r="H303" s="5" t="s">
         <v>969</v>
@@ -17038,7 +17036,7 @@
         <v>73</v>
       </c>
       <c r="J303" s="3" t="s">
-        <v>1429</v>
+        <v>1427</v>
       </c>
       <c r="L303" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17063,16 +17061,16 @@
         <v>432</v>
       </c>
       <c r="E304" s="3" t="s">
+        <v>1428</v>
+      </c>
+      <c r="F304" s="3" t="s">
+        <v>1429</v>
+      </c>
+      <c r="H304" s="5" t="s">
         <v>1430</v>
       </c>
-      <c r="F304" s="3" t="s">
+      <c r="J304" s="3" t="s">
         <v>1431</v>
-      </c>
-      <c r="H304" s="5" t="s">
-        <v>1432</v>
-      </c>
-      <c r="J304" s="3" t="s">
-        <v>1433</v>
       </c>
       <c r="L304" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17097,13 +17095,13 @@
         <v>365</v>
       </c>
       <c r="E305" s="3" t="s">
-        <v>1434</v>
+        <v>1432</v>
       </c>
       <c r="F305" s="5" t="s">
         <v>439</v>
       </c>
       <c r="G305" s="5" t="s">
-        <v>1435</v>
+        <v>1433</v>
       </c>
       <c r="H305" s="5" t="s">
         <v>1049</v>
@@ -17137,16 +17135,16 @@
         <v>445</v>
       </c>
       <c r="E306" s="3" t="s">
-        <v>1436</v>
+        <v>1434</v>
       </c>
       <c r="F306" s="3" t="s">
-        <v>1437</v>
+        <v>1435</v>
       </c>
       <c r="H306" s="5" t="s">
         <v>1054</v>
       </c>
       <c r="J306" s="3" t="s">
-        <v>1438</v>
+        <v>1436</v>
       </c>
       <c r="L306" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17171,7 +17169,7 @@
         <v>200</v>
       </c>
       <c r="E307" s="3" t="s">
-        <v>1439</v>
+        <v>1437</v>
       </c>
       <c r="F307" s="3" t="s">
         <v>452</v>
@@ -17208,7 +17206,7 @@
         <v>372</v>
       </c>
       <c r="E308" s="3" t="s">
-        <v>1440</v>
+        <v>1438</v>
       </c>
       <c r="F308" s="3" t="s">
         <v>457</v>
@@ -17220,7 +17218,7 @@
         <v>459</v>
       </c>
       <c r="J308" s="3" t="s">
-        <v>1441</v>
+        <v>1439</v>
       </c>
       <c r="L308" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17245,10 +17243,10 @@
         <v>21</v>
       </c>
       <c r="E309" s="3" t="s">
-        <v>1442</v>
+        <v>1440</v>
       </c>
       <c r="F309" s="3" t="s">
-        <v>1443</v>
+        <v>1441</v>
       </c>
       <c r="H309" s="5" t="s">
         <v>1063</v>
@@ -17279,7 +17277,7 @@
         <v>153</v>
       </c>
       <c r="E310" s="3" t="s">
-        <v>1444</v>
+        <v>1442</v>
       </c>
       <c r="F310" s="3" t="s">
         <v>1067</v>
@@ -17288,7 +17286,7 @@
         <v>1068</v>
       </c>
       <c r="J310" s="3" t="s">
-        <v>1445</v>
+        <v>1443</v>
       </c>
       <c r="L310" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17313,22 +17311,22 @@
         <v>471</v>
       </c>
       <c r="E311" s="3" t="s">
+        <v>1444</v>
+      </c>
+      <c r="F311" s="3" t="s">
+        <v>1445</v>
+      </c>
+      <c r="G311" s="3" t="s">
         <v>1446</v>
       </c>
-      <c r="F311" s="3" t="s">
+      <c r="H311" s="5" t="s">
         <v>1447</v>
       </c>
-      <c r="G311" s="3" t="s">
+      <c r="I311" s="3" t="s">
         <v>1448</v>
       </c>
-      <c r="H311" s="5" t="s">
+      <c r="J311" s="3" t="s">
         <v>1449</v>
-      </c>
-      <c r="I311" s="3" t="s">
-        <v>1450</v>
-      </c>
-      <c r="J311" s="3" t="s">
-        <v>1451</v>
       </c>
       <c r="L311" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17353,7 +17351,7 @@
         <v>123</v>
       </c>
       <c r="E312" s="3" t="s">
-        <v>1452</v>
+        <v>1450</v>
       </c>
       <c r="F312" s="3" t="s">
         <v>485</v>
@@ -17387,7 +17385,7 @@
         <v>445</v>
       </c>
       <c r="E313" s="3" t="s">
-        <v>1453</v>
+        <v>1451</v>
       </c>
       <c r="F313" s="3" t="s">
         <v>490</v>
@@ -17399,7 +17397,7 @@
         <v>492</v>
       </c>
       <c r="J313" s="3" t="s">
-        <v>1454</v>
+        <v>1452</v>
       </c>
       <c r="L313" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17424,7 +17422,7 @@
         <v>495</v>
       </c>
       <c r="E314" s="3" t="s">
-        <v>1455</v>
+        <v>1453</v>
       </c>
       <c r="F314" s="3" t="s">
         <v>497</v>
@@ -17433,7 +17431,7 @@
         <v>1093</v>
       </c>
       <c r="J314" s="3" t="s">
-        <v>1456</v>
+        <v>1454</v>
       </c>
       <c r="L314" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17458,16 +17456,16 @@
         <v>501</v>
       </c>
       <c r="E315" s="3" t="s">
-        <v>1457</v>
+        <v>1455</v>
       </c>
       <c r="F315" s="3" t="s">
-        <v>1458</v>
+        <v>1456</v>
       </c>
       <c r="H315" s="5" t="s">
         <v>1098</v>
       </c>
       <c r="J315" s="3" t="s">
-        <v>1459</v>
+        <v>1457</v>
       </c>
       <c r="L315" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17492,7 +17490,7 @@
         <v>29</v>
       </c>
       <c r="E316" s="3" t="s">
-        <v>1460</v>
+        <v>1458</v>
       </c>
       <c r="F316" s="3" t="s">
         <v>509</v>
@@ -17529,7 +17527,7 @@
         <v>515</v>
       </c>
       <c r="E317" s="3" t="s">
-        <v>1461</v>
+        <v>1459</v>
       </c>
       <c r="F317" s="3" t="s">
         <v>517</v>
@@ -17563,7 +17561,7 @@
         <v>521</v>
       </c>
       <c r="E318" s="3" t="s">
-        <v>1462</v>
+        <v>1460</v>
       </c>
       <c r="F318" s="3" t="s">
         <v>523</v>
@@ -17600,10 +17598,10 @@
         <v>528</v>
       </c>
       <c r="E319" s="3" t="s">
-        <v>1463</v>
+        <v>1461</v>
       </c>
       <c r="F319" s="3" t="s">
-        <v>1464</v>
+        <v>1462</v>
       </c>
       <c r="H319" s="5" t="s">
         <v>1120</v>
@@ -17637,7 +17635,7 @@
         <v>536</v>
       </c>
       <c r="E320" s="3" t="s">
-        <v>1465</v>
+        <v>1463</v>
       </c>
       <c r="F320" s="3" t="s">
         <v>538</v>
@@ -17646,7 +17644,7 @@
         <v>1123</v>
       </c>
       <c r="J320" s="3" t="s">
-        <v>1466</v>
+        <v>1464</v>
       </c>
       <c r="L320" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17671,16 +17669,16 @@
         <v>543</v>
       </c>
       <c r="E321" s="3" t="s">
-        <v>1467</v>
+        <v>1465</v>
       </c>
       <c r="F321" s="3" t="s">
-        <v>1468</v>
+        <v>1466</v>
       </c>
       <c r="H321" s="5" t="s">
         <v>1127</v>
       </c>
       <c r="J321" s="3" t="s">
-        <v>1469</v>
+        <v>1467</v>
       </c>
       <c r="L321" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17705,7 +17703,7 @@
         <v>550</v>
       </c>
       <c r="E322" s="3" t="s">
-        <v>1470</v>
+        <v>1468</v>
       </c>
       <c r="F322" s="3" t="s">
         <v>552</v>
@@ -17717,7 +17715,7 @@
         <v>73</v>
       </c>
       <c r="J322" s="3" t="s">
-        <v>1471</v>
+        <v>1469</v>
       </c>
       <c r="L322" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17742,19 +17740,19 @@
         <v>556</v>
       </c>
       <c r="E323" s="3" t="s">
-        <v>1472</v>
+        <v>1470</v>
       </c>
       <c r="F323" s="3" t="s">
-        <v>1473</v>
+        <v>1471</v>
       </c>
       <c r="H323" s="5" t="s">
         <v>1266</v>
       </c>
       <c r="I323" s="3" t="s">
-        <v>1474</v>
+        <v>1472</v>
       </c>
       <c r="J323" s="3" t="s">
-        <v>1451</v>
+        <v>1449</v>
       </c>
       <c r="L323" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17779,13 +17777,13 @@
         <v>391</v>
       </c>
       <c r="E324" s="3" t="s">
+        <v>1473</v>
+      </c>
+      <c r="F324" s="3" t="s">
+        <v>1474</v>
+      </c>
+      <c r="G324" s="3" t="s">
         <v>1475</v>
-      </c>
-      <c r="F324" s="3" t="s">
-        <v>1476</v>
-      </c>
-      <c r="G324" s="3" t="s">
-        <v>1477</v>
       </c>
       <c r="H324" s="5" t="s">
         <v>1298</v>
@@ -17810,22 +17808,22 @@
         <v>19</v>
       </c>
       <c r="C325" s="3" t="s">
+        <v>1476</v>
+      </c>
+      <c r="E325" s="3" t="s">
+        <v>1477</v>
+      </c>
+      <c r="F325" s="3" t="s">
         <v>1478</v>
-      </c>
-      <c r="E325" s="3" t="s">
-        <v>1479</v>
-      </c>
-      <c r="F325" s="3" t="s">
-        <v>1480</v>
       </c>
       <c r="H325" s="3" t="s">
         <v>571</v>
       </c>
       <c r="I325" s="3" t="s">
-        <v>1481</v>
+        <v>1479</v>
       </c>
       <c r="J325" s="3" t="s">
-        <v>1482</v>
+        <v>1480</v>
       </c>
       <c r="L325" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17844,10 +17842,10 @@
         <v>28</v>
       </c>
       <c r="C326" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E326" s="3" t="s">
-        <v>1483</v>
+        <v>1481</v>
       </c>
       <c r="F326" s="3" t="s">
         <v>575</v>
@@ -17856,10 +17854,10 @@
         <v>576</v>
       </c>
       <c r="I326" s="3" t="s">
-        <v>1484</v>
+        <v>1482</v>
       </c>
       <c r="J326" s="3" t="s">
-        <v>1485</v>
+        <v>1483</v>
       </c>
       <c r="L326" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17878,10 +17876,10 @@
         <v>34</v>
       </c>
       <c r="C327" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E327" s="3" t="s">
-        <v>1486</v>
+        <v>1484</v>
       </c>
       <c r="F327" s="3" t="s">
         <v>37</v>
@@ -17893,7 +17891,7 @@
         <v>39</v>
       </c>
       <c r="J327" s="3" t="s">
-        <v>1487</v>
+        <v>1485</v>
       </c>
       <c r="L327" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17912,10 +17910,10 @@
         <v>41</v>
       </c>
       <c r="C328" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E328" s="3" t="s">
-        <v>1488</v>
+        <v>1486</v>
       </c>
       <c r="F328" s="3" t="s">
         <v>1307</v>
@@ -17924,10 +17922,10 @@
         <v>584</v>
       </c>
       <c r="I328" s="3" t="s">
-        <v>1489</v>
+        <v>1487</v>
       </c>
       <c r="J328" s="3" t="s">
-        <v>1490</v>
+        <v>1488</v>
       </c>
       <c r="L328" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17946,10 +17944,10 @@
         <v>48</v>
       </c>
       <c r="C329" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E329" s="3" t="s">
-        <v>1491</v>
+        <v>1489</v>
       </c>
       <c r="F329" s="3" t="s">
         <v>51</v>
@@ -17958,10 +17956,10 @@
         <v>589</v>
       </c>
       <c r="I329" s="3" t="s">
-        <v>1492</v>
+        <v>1490</v>
       </c>
       <c r="J329" s="3" t="s">
-        <v>1493</v>
+        <v>1491</v>
       </c>
       <c r="L329" s="3" t="str">
         <f t="shared" si="3"/>
@@ -17980,10 +17978,10 @@
         <v>56</v>
       </c>
       <c r="C330" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E330" s="3" t="s">
-        <v>1494</v>
+        <v>1492</v>
       </c>
       <c r="F330" s="3" t="s">
         <v>57</v>
@@ -17995,7 +17993,7 @@
         <v>59</v>
       </c>
       <c r="J330" s="3" t="s">
-        <v>1495</v>
+        <v>1493</v>
       </c>
       <c r="L330" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18014,10 +18012,10 @@
         <v>61</v>
       </c>
       <c r="C331" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E331" s="3" t="s">
-        <v>1496</v>
+        <v>1494</v>
       </c>
       <c r="F331" s="3" t="s">
         <v>597</v>
@@ -18029,7 +18027,7 @@
         <v>66</v>
       </c>
       <c r="J331" s="3" t="s">
-        <v>1497</v>
+        <v>1495</v>
       </c>
       <c r="L331" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18048,22 +18046,22 @@
         <v>68</v>
       </c>
       <c r="C332" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E332" s="3" t="s">
-        <v>1498</v>
+        <v>1496</v>
       </c>
       <c r="F332" s="3" t="s">
-        <v>1499</v>
+        <v>1497</v>
       </c>
       <c r="H332" s="3" t="s">
         <v>603</v>
       </c>
       <c r="I332" s="3" t="s">
-        <v>1500</v>
+        <v>1498</v>
       </c>
       <c r="J332" s="3" t="s">
-        <v>1501</v>
+        <v>1499</v>
       </c>
       <c r="L332" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18082,10 +18080,10 @@
         <v>75</v>
       </c>
       <c r="C333" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E333" s="3" t="s">
-        <v>1502</v>
+        <v>1500</v>
       </c>
       <c r="F333" s="3" t="s">
         <v>78</v>
@@ -18094,7 +18092,7 @@
         <v>607</v>
       </c>
       <c r="J333" s="3" t="s">
-        <v>1503</v>
+        <v>1501</v>
       </c>
       <c r="L333" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18113,10 +18111,10 @@
         <v>81</v>
       </c>
       <c r="C334" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E334" s="3" t="s">
-        <v>1504</v>
+        <v>1502</v>
       </c>
       <c r="F334" s="3" t="s">
         <v>84</v>
@@ -18125,10 +18123,10 @@
         <v>612</v>
       </c>
       <c r="I334" s="3" t="s">
-        <v>1505</v>
+        <v>1503</v>
       </c>
       <c r="J334" s="3" t="s">
-        <v>1506</v>
+        <v>1504</v>
       </c>
       <c r="L334" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18147,10 +18145,10 @@
         <v>87</v>
       </c>
       <c r="C335" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E335" s="3" t="s">
-        <v>1507</v>
+        <v>1505</v>
       </c>
       <c r="F335" s="3" t="s">
         <v>90</v>
@@ -18162,7 +18160,7 @@
         <v>92</v>
       </c>
       <c r="J335" s="3" t="s">
-        <v>1508</v>
+        <v>1506</v>
       </c>
       <c r="L335" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18181,10 +18179,10 @@
         <v>94</v>
       </c>
       <c r="C336" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E336" s="3" t="s">
-        <v>1509</v>
+        <v>1507</v>
       </c>
       <c r="F336" s="3" t="s">
         <v>97</v>
@@ -18196,7 +18194,7 @@
         <v>99</v>
       </c>
       <c r="J336" s="3" t="s">
-        <v>1510</v>
+        <v>1508</v>
       </c>
       <c r="L336" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18215,10 +18213,10 @@
         <v>101</v>
       </c>
       <c r="C337" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E337" s="3" t="s">
-        <v>1511</v>
+        <v>1509</v>
       </c>
       <c r="F337" s="3" t="s">
         <v>104</v>
@@ -18230,7 +18228,7 @@
         <v>106</v>
       </c>
       <c r="J337" s="3" t="s">
-        <v>1512</v>
+        <v>1510</v>
       </c>
       <c r="L337" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18249,10 +18247,10 @@
         <v>108</v>
       </c>
       <c r="C338" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E338" s="3" t="s">
-        <v>1513</v>
+        <v>1511</v>
       </c>
       <c r="F338" s="3" t="s">
         <v>111</v>
@@ -18264,7 +18262,7 @@
         <v>113</v>
       </c>
       <c r="J338" s="3" t="s">
-        <v>1514</v>
+        <v>1512</v>
       </c>
       <c r="L338" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18283,10 +18281,10 @@
         <v>115</v>
       </c>
       <c r="C339" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E339" s="3" t="s">
-        <v>1515</v>
+        <v>1513</v>
       </c>
       <c r="F339" s="3" t="s">
         <v>118</v>
@@ -18298,7 +18296,7 @@
         <v>120</v>
       </c>
       <c r="J339" s="3" t="s">
-        <v>1516</v>
+        <v>1514</v>
       </c>
       <c r="L339" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18317,10 +18315,10 @@
         <v>122</v>
       </c>
       <c r="C340" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E340" s="3" t="s">
-        <v>1517</v>
+        <v>1515</v>
       </c>
       <c r="F340" s="3" t="s">
         <v>125</v>
@@ -18329,10 +18327,10 @@
         <v>642</v>
       </c>
       <c r="I340" s="3" t="s">
-        <v>1518</v>
+        <v>1516</v>
       </c>
       <c r="J340" s="3" t="s">
-        <v>1519</v>
+        <v>1517</v>
       </c>
       <c r="L340" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18351,22 +18349,22 @@
         <v>130</v>
       </c>
       <c r="C341" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E341" s="3" t="s">
-        <v>1520</v>
+        <v>1518</v>
       </c>
       <c r="F341" s="3" t="s">
         <v>133</v>
       </c>
       <c r="H341" s="3" t="s">
-        <v>1521</v>
+        <v>1519</v>
       </c>
       <c r="I341" s="3" t="s">
         <v>135</v>
       </c>
       <c r="J341" s="3" t="s">
-        <v>1522</v>
+        <v>1520</v>
       </c>
       <c r="L341" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18385,10 +18383,10 @@
         <v>137</v>
       </c>
       <c r="C342" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E342" s="3" t="s">
-        <v>1523</v>
+        <v>1521</v>
       </c>
       <c r="F342" s="3" t="s">
         <v>651</v>
@@ -18400,7 +18398,7 @@
         <v>142</v>
       </c>
       <c r="J342" s="3" t="s">
-        <v>1524</v>
+        <v>1522</v>
       </c>
       <c r="L342" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18419,10 +18417,10 @@
         <v>144</v>
       </c>
       <c r="C343" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E343" s="3" t="s">
-        <v>1525</v>
+        <v>1523</v>
       </c>
       <c r="F343" s="3" t="s">
         <v>147</v>
@@ -18434,7 +18432,7 @@
         <v>150</v>
       </c>
       <c r="J343" s="3" t="s">
-        <v>1526</v>
+        <v>1524</v>
       </c>
       <c r="L343" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18453,10 +18451,10 @@
         <v>152</v>
       </c>
       <c r="C344" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E344" s="3" t="s">
-        <v>1527</v>
+        <v>1525</v>
       </c>
       <c r="F344" s="3" t="s">
         <v>155</v>
@@ -18468,7 +18466,7 @@
         <v>157</v>
       </c>
       <c r="J344" s="3" t="s">
-        <v>1528</v>
+        <v>1526</v>
       </c>
       <c r="L344" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18487,10 +18485,10 @@
         <v>159</v>
       </c>
       <c r="C345" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E345" s="3" t="s">
-        <v>1529</v>
+        <v>1527</v>
       </c>
       <c r="F345" s="3" t="s">
         <v>162</v>
@@ -18502,7 +18500,7 @@
         <v>164</v>
       </c>
       <c r="J345" s="3" t="s">
-        <v>1530</v>
+        <v>1528</v>
       </c>
       <c r="L345" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18521,13 +18519,13 @@
         <v>166</v>
       </c>
       <c r="C346" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E346" s="3" t="s">
-        <v>1531</v>
+        <v>1529</v>
       </c>
       <c r="F346" s="3" t="s">
-        <v>1532</v>
+        <v>1530</v>
       </c>
       <c r="H346" s="3" t="s">
         <v>670</v>
@@ -18536,7 +18534,7 @@
         <v>172</v>
       </c>
       <c r="J346" s="3" t="s">
-        <v>1533</v>
+        <v>1531</v>
       </c>
       <c r="L346" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18555,10 +18553,10 @@
         <v>174</v>
       </c>
       <c r="C347" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E347" s="3" t="s">
-        <v>1534</v>
+        <v>1532</v>
       </c>
       <c r="F347" s="3" t="s">
         <v>177</v>
@@ -18570,7 +18568,7 @@
         <v>179</v>
       </c>
       <c r="J347" s="3" t="s">
-        <v>1535</v>
+        <v>1533</v>
       </c>
       <c r="L347" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18589,22 +18587,22 @@
         <v>181</v>
       </c>
       <c r="C348" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E348" s="3" t="s">
-        <v>1536</v>
+        <v>1534</v>
       </c>
       <c r="F348" s="3" t="s">
-        <v>1537</v>
+        <v>1535</v>
       </c>
       <c r="H348" s="3" t="s">
         <v>676</v>
       </c>
       <c r="I348" s="3" t="s">
-        <v>1538</v>
+        <v>1536</v>
       </c>
       <c r="J348" s="3" t="s">
-        <v>1539</v>
+        <v>1537</v>
       </c>
       <c r="L348" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18623,19 +18621,19 @@
         <v>188</v>
       </c>
       <c r="C349" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E349" s="3" t="s">
-        <v>1540</v>
+        <v>1538</v>
       </c>
       <c r="F349" s="3" t="s">
-        <v>1541</v>
+        <v>1539</v>
       </c>
       <c r="H349" s="3" t="s">
         <v>682</v>
       </c>
       <c r="J349" s="3" t="s">
-        <v>1542</v>
+        <v>1540</v>
       </c>
       <c r="L349" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18654,13 +18652,13 @@
         <v>195</v>
       </c>
       <c r="C350" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E350" s="3" t="s">
-        <v>1543</v>
+        <v>1541</v>
       </c>
       <c r="F350" s="3" t="s">
-        <v>1544</v>
+        <v>1542</v>
       </c>
       <c r="H350" s="3" t="s">
         <v>722</v>
@@ -18669,7 +18667,7 @@
         <v>198</v>
       </c>
       <c r="J350" s="3" t="s">
-        <v>1545</v>
+        <v>1543</v>
       </c>
       <c r="L350" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18688,10 +18686,10 @@
         <v>199</v>
       </c>
       <c r="C351" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E351" s="3" t="s">
-        <v>1546</v>
+        <v>1544</v>
       </c>
       <c r="F351" s="3" t="s">
         <v>202</v>
@@ -18703,7 +18701,7 @@
         <v>204</v>
       </c>
       <c r="J351" s="3" t="s">
-        <v>1547</v>
+        <v>1545</v>
       </c>
       <c r="L351" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18722,10 +18720,10 @@
         <v>207</v>
       </c>
       <c r="C352" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E352" s="3" t="s">
-        <v>1548</v>
+        <v>1546</v>
       </c>
       <c r="F352" s="3" t="s">
         <v>728</v>
@@ -18734,10 +18732,10 @@
         <v>729</v>
       </c>
       <c r="I352" s="3" t="s">
-        <v>1549</v>
+        <v>1547</v>
       </c>
       <c r="J352" s="3" t="s">
-        <v>1550</v>
+        <v>1548</v>
       </c>
       <c r="L352" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18756,13 +18754,13 @@
         <v>212</v>
       </c>
       <c r="C353" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E353" s="3" t="s">
-        <v>1551</v>
+        <v>1549</v>
       </c>
       <c r="F353" s="3" t="s">
-        <v>1552</v>
+        <v>1550</v>
       </c>
       <c r="H353" s="3" t="s">
         <v>734</v>
@@ -18771,7 +18769,7 @@
         <v>216</v>
       </c>
       <c r="J353" s="3" t="s">
-        <v>1553</v>
+        <v>1551</v>
       </c>
       <c r="L353" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18790,10 +18788,10 @@
         <v>218</v>
       </c>
       <c r="C354" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E354" s="3" t="s">
-        <v>1554</v>
+        <v>1552</v>
       </c>
       <c r="F354" s="3" t="s">
         <v>221</v>
@@ -18802,10 +18800,10 @@
         <v>739</v>
       </c>
       <c r="I354" s="3" t="s">
-        <v>1555</v>
+        <v>1553</v>
       </c>
       <c r="J354" s="3" t="s">
-        <v>1556</v>
+        <v>1554</v>
       </c>
       <c r="L354" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18824,10 +18822,10 @@
         <v>224</v>
       </c>
       <c r="C355" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E355" s="3" t="s">
-        <v>1557</v>
+        <v>1555</v>
       </c>
       <c r="F355" s="3" t="s">
         <v>225</v>
@@ -18839,7 +18837,7 @@
         <v>227</v>
       </c>
       <c r="J355" s="3" t="s">
-        <v>1558</v>
+        <v>1556</v>
       </c>
       <c r="L355" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18858,10 +18856,10 @@
         <v>229</v>
       </c>
       <c r="C356" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E356" s="3" t="s">
-        <v>1559</v>
+        <v>1557</v>
       </c>
       <c r="F356" s="3" t="s">
         <v>746</v>
@@ -18873,7 +18871,7 @@
         <v>234</v>
       </c>
       <c r="J356" s="3" t="s">
-        <v>1560</v>
+        <v>1558</v>
       </c>
       <c r="L356" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18892,10 +18890,10 @@
         <v>236</v>
       </c>
       <c r="C357" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E357" s="3" t="s">
-        <v>1561</v>
+        <v>1559</v>
       </c>
       <c r="F357" s="3" t="s">
         <v>239</v>
@@ -18907,7 +18905,7 @@
         <v>242</v>
       </c>
       <c r="J357" s="3" t="s">
-        <v>1562</v>
+        <v>1560</v>
       </c>
       <c r="L357" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18926,10 +18924,10 @@
         <v>244</v>
       </c>
       <c r="C358" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E358" s="3" t="s">
-        <v>1563</v>
+        <v>1561</v>
       </c>
       <c r="F358" s="3" t="s">
         <v>247</v>
@@ -18941,7 +18939,7 @@
         <v>249</v>
       </c>
       <c r="J358" s="3" t="s">
-        <v>1564</v>
+        <v>1562</v>
       </c>
       <c r="L358" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18960,10 +18958,10 @@
         <v>251</v>
       </c>
       <c r="C359" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E359" s="3" t="s">
-        <v>1565</v>
+        <v>1563</v>
       </c>
       <c r="F359" s="3" t="s">
         <v>252</v>
@@ -18975,7 +18973,7 @@
         <v>255</v>
       </c>
       <c r="J359" s="3" t="s">
-        <v>1566</v>
+        <v>1564</v>
       </c>
       <c r="L359" s="3" t="str">
         <f t="shared" si="3"/>
@@ -18994,13 +18992,13 @@
         <v>258</v>
       </c>
       <c r="C360" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E360" s="3" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
       <c r="F360" s="3" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="H360" s="3" t="s">
         <v>775</v>
@@ -19028,10 +19026,10 @@
         <v>263</v>
       </c>
       <c r="C361" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E361" s="3" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
       <c r="F361" s="3" t="s">
         <v>266</v>
@@ -19040,7 +19038,7 @@
         <v>779</v>
       </c>
       <c r="I361" s="3" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
       <c r="J361" s="3" t="s">
         <v>269</v>
@@ -19062,10 +19060,10 @@
         <v>270</v>
       </c>
       <c r="C362" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E362" s="3" t="s">
-        <v>1571</v>
+        <v>1569</v>
       </c>
       <c r="F362" s="3" t="s">
         <v>273</v>
@@ -19074,10 +19072,10 @@
         <v>781</v>
       </c>
       <c r="I362" s="3" t="s">
-        <v>1572</v>
+        <v>1570</v>
       </c>
       <c r="J362" s="3" t="s">
-        <v>1573</v>
+        <v>1571</v>
       </c>
       <c r="L362" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19096,22 +19094,22 @@
         <v>277</v>
       </c>
       <c r="C363" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E363" s="3" t="s">
+        <v>1572</v>
+      </c>
+      <c r="F363" s="3" t="s">
+        <v>1378</v>
+      </c>
+      <c r="H363" s="3" t="s">
+        <v>1379</v>
+      </c>
+      <c r="I363" s="3" t="s">
+        <v>1573</v>
+      </c>
+      <c r="J363" s="3" t="s">
         <v>1574</v>
-      </c>
-      <c r="F363" s="3" t="s">
-        <v>1380</v>
-      </c>
-      <c r="H363" s="3" t="s">
-        <v>1381</v>
-      </c>
-      <c r="I363" s="3" t="s">
-        <v>1575</v>
-      </c>
-      <c r="J363" s="3" t="s">
-        <v>1576</v>
       </c>
       <c r="L363" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19130,19 +19128,19 @@
         <v>284</v>
       </c>
       <c r="C364" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E364" s="3" t="s">
-        <v>1577</v>
+        <v>1575</v>
       </c>
       <c r="F364" s="3" t="s">
-        <v>1578</v>
+        <v>1576</v>
       </c>
       <c r="H364" s="3" t="s">
         <v>791</v>
       </c>
       <c r="I364" s="3" t="s">
-        <v>1579</v>
+        <v>1577</v>
       </c>
       <c r="J364" s="3" t="s">
         <v>289</v>
@@ -19164,10 +19162,10 @@
         <v>290</v>
       </c>
       <c r="C365" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E365" s="3" t="s">
-        <v>1580</v>
+        <v>1578</v>
       </c>
       <c r="F365" s="3" t="s">
         <v>293</v>
@@ -19179,7 +19177,7 @@
         <v>295</v>
       </c>
       <c r="J365" s="3" t="s">
-        <v>1581</v>
+        <v>1579</v>
       </c>
       <c r="L365" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19198,22 +19196,22 @@
         <v>297</v>
       </c>
       <c r="C366" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E366" s="3" t="s">
-        <v>1582</v>
+        <v>1580</v>
       </c>
       <c r="F366" s="3" t="s">
         <v>298</v>
       </c>
       <c r="H366" s="3" t="s">
-        <v>1583</v>
+        <v>1581</v>
       </c>
       <c r="I366" s="3" t="s">
         <v>300</v>
       </c>
       <c r="J366" s="3" t="s">
-        <v>1584</v>
+        <v>1582</v>
       </c>
       <c r="L366" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19232,10 +19230,10 @@
         <v>302</v>
       </c>
       <c r="C367" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E367" s="3" t="s">
-        <v>1585</v>
+        <v>1583</v>
       </c>
       <c r="F367" s="3" t="s">
         <v>305</v>
@@ -19263,10 +19261,10 @@
         <v>309</v>
       </c>
       <c r="C368" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E368" s="3" t="s">
-        <v>1586</v>
+        <v>1584</v>
       </c>
       <c r="F368" s="3" t="s">
         <v>312</v>
@@ -19278,7 +19276,7 @@
         <v>314</v>
       </c>
       <c r="J368" s="3" t="s">
-        <v>1587</v>
+        <v>1585</v>
       </c>
       <c r="L368" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19297,16 +19295,16 @@
         <v>316</v>
       </c>
       <c r="C369" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E369" s="3" t="s">
-        <v>1588</v>
+        <v>1586</v>
       </c>
       <c r="F369" s="3" t="s">
         <v>317</v>
       </c>
       <c r="H369" s="3" t="s">
-        <v>1589</v>
+        <v>1587</v>
       </c>
       <c r="J369" s="3" t="s">
         <v>320</v>
@@ -19328,10 +19326,10 @@
         <v>321</v>
       </c>
       <c r="C370" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E370" s="3" t="s">
-        <v>1590</v>
+        <v>1588</v>
       </c>
       <c r="F370" s="3" t="s">
         <v>324</v>
@@ -19343,7 +19341,7 @@
         <v>326</v>
       </c>
       <c r="J370" s="3" t="s">
-        <v>1591</v>
+        <v>1589</v>
       </c>
       <c r="L370" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19362,10 +19360,10 @@
         <v>328</v>
       </c>
       <c r="C371" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E371" s="3" t="s">
-        <v>1592</v>
+        <v>1590</v>
       </c>
       <c r="F371" s="3" t="s">
         <v>331</v>
@@ -19374,10 +19372,10 @@
         <v>843</v>
       </c>
       <c r="I371" s="3" t="s">
-        <v>1593</v>
+        <v>1591</v>
       </c>
       <c r="J371" s="3" t="s">
-        <v>1594</v>
+        <v>1592</v>
       </c>
       <c r="L371" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19396,10 +19394,10 @@
         <v>335</v>
       </c>
       <c r="C372" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E372" s="3" t="s">
-        <v>1595</v>
+        <v>1593</v>
       </c>
       <c r="F372" s="3" t="s">
         <v>847</v>
@@ -19408,10 +19406,10 @@
         <v>848</v>
       </c>
       <c r="I372" s="3" t="s">
-        <v>1596</v>
+        <v>1594</v>
       </c>
       <c r="J372" s="3" t="s">
-        <v>1597</v>
+        <v>1595</v>
       </c>
       <c r="L372" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19430,13 +19428,13 @@
         <v>340</v>
       </c>
       <c r="C373" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E373" s="3" t="s">
-        <v>1598</v>
+        <v>1596</v>
       </c>
       <c r="F373" s="3" t="s">
-        <v>1599</v>
+        <v>1597</v>
       </c>
       <c r="H373" s="3" t="s">
         <v>850</v>
@@ -19445,7 +19443,7 @@
         <v>343</v>
       </c>
       <c r="J373" s="3" t="s">
-        <v>1600</v>
+        <v>1598</v>
       </c>
       <c r="L373" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19464,20 +19462,20 @@
         <v>345</v>
       </c>
       <c r="C374" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E374" s="3" t="s">
-        <v>1601</v>
+        <v>1599</v>
       </c>
       <c r="F374" s="3" t="s">
-        <v>1602</v>
+        <v>1600</v>
       </c>
       <c r="H374" s="3" t="s">
-        <v>1401</v>
+        <v>1399</v>
       </c>
       <c r="I374" s="3"/>
       <c r="J374" s="3" t="s">
-        <v>1603</v>
+        <v>1601</v>
       </c>
       <c r="L374" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19496,22 +19494,22 @@
         <v>352</v>
       </c>
       <c r="C375" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E375" s="3" t="s">
-        <v>1604</v>
+        <v>1602</v>
       </c>
       <c r="F375" s="3" t="s">
-        <v>1605</v>
+        <v>1603</v>
       </c>
       <c r="H375" s="3" t="s">
         <v>912</v>
       </c>
       <c r="I375" s="3" t="s">
-        <v>1606</v>
+        <v>1604</v>
       </c>
       <c r="J375" s="3" t="s">
-        <v>1607</v>
+        <v>1605</v>
       </c>
       <c r="L375" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19530,10 +19528,10 @@
         <v>357</v>
       </c>
       <c r="C376" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E376" s="3" t="s">
-        <v>1608</v>
+        <v>1606</v>
       </c>
       <c r="F376" s="3" t="s">
         <v>360</v>
@@ -19542,10 +19540,10 @@
         <v>923</v>
       </c>
       <c r="I376" s="3" t="s">
-        <v>1609</v>
+        <v>1607</v>
       </c>
       <c r="J376" s="3" t="s">
-        <v>1610</v>
+        <v>1608</v>
       </c>
       <c r="L376" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19564,10 +19562,10 @@
         <v>364</v>
       </c>
       <c r="C377" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E377" s="3" t="s">
-        <v>1611</v>
+        <v>1609</v>
       </c>
       <c r="F377" s="3" t="s">
         <v>367</v>
@@ -19579,7 +19577,7 @@
         <v>369</v>
       </c>
       <c r="J377" s="3" t="s">
-        <v>1612</v>
+        <v>1610</v>
       </c>
       <c r="L377" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19598,13 +19596,13 @@
         <v>371</v>
       </c>
       <c r="C378" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E378" s="3" t="s">
-        <v>1613</v>
+        <v>1611</v>
       </c>
       <c r="F378" s="3" t="s">
-        <v>1614</v>
+        <v>1612</v>
       </c>
       <c r="H378" s="3" t="s">
         <v>932</v>
@@ -19613,7 +19611,7 @@
         <v>376</v>
       </c>
       <c r="J378" s="3" t="s">
-        <v>1615</v>
+        <v>1613</v>
       </c>
       <c r="L378" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19632,13 +19630,13 @@
         <v>378</v>
       </c>
       <c r="C379" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E379" s="3" t="s">
-        <v>1616</v>
+        <v>1614</v>
       </c>
       <c r="F379" s="3" t="s">
-        <v>1410</v>
+        <v>1408</v>
       </c>
       <c r="H379" s="3" t="s">
         <v>936</v>
@@ -19647,7 +19645,7 @@
         <v>381</v>
       </c>
       <c r="J379" s="3" t="s">
-        <v>1617</v>
+        <v>1615</v>
       </c>
       <c r="L379" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19666,13 +19664,13 @@
         <v>383</v>
       </c>
       <c r="C380" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E380" s="3" t="s">
-        <v>1618</v>
+        <v>1616</v>
       </c>
       <c r="F380" s="3" t="s">
-        <v>1619</v>
+        <v>1617</v>
       </c>
       <c r="H380" s="3" t="s">
         <v>940</v>
@@ -19681,7 +19679,7 @@
         <v>388</v>
       </c>
       <c r="J380" s="3" t="s">
-        <v>1620</v>
+        <v>1618</v>
       </c>
       <c r="L380" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19700,19 +19698,19 @@
         <v>390</v>
       </c>
       <c r="C381" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E381" s="3" t="s">
-        <v>1621</v>
+        <v>1619</v>
       </c>
       <c r="F381" s="3" t="s">
-        <v>1622</v>
+        <v>1620</v>
       </c>
       <c r="H381" s="3" t="s">
         <v>945</v>
       </c>
       <c r="J381" s="3" t="s">
-        <v>1623</v>
+        <v>1621</v>
       </c>
       <c r="L381" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19731,10 +19729,10 @@
         <v>398</v>
       </c>
       <c r="C382" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E382" s="3" t="s">
-        <v>1624</v>
+        <v>1622</v>
       </c>
       <c r="F382" s="3" t="s">
         <v>401</v>
@@ -19746,7 +19744,7 @@
         <v>403</v>
       </c>
       <c r="J382" s="3" t="s">
-        <v>1625</v>
+        <v>1623</v>
       </c>
       <c r="L382" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19765,13 +19763,13 @@
         <v>405</v>
       </c>
       <c r="C383" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E383" s="3" t="s">
-        <v>1626</v>
+        <v>1624</v>
       </c>
       <c r="F383" s="3" t="s">
-        <v>1627</v>
+        <v>1625</v>
       </c>
       <c r="H383" s="3" t="s">
         <v>959</v>
@@ -19780,7 +19778,7 @@
         <v>409</v>
       </c>
       <c r="J383" s="3" t="s">
-        <v>1628</v>
+        <v>1626</v>
       </c>
       <c r="L383" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19799,10 +19797,10 @@
         <v>411</v>
       </c>
       <c r="C384" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E384" s="3" t="s">
-        <v>1629</v>
+        <v>1627</v>
       </c>
       <c r="F384" s="3" t="s">
         <v>412</v>
@@ -19814,7 +19812,7 @@
         <v>415</v>
       </c>
       <c r="J384" s="3" t="s">
-        <v>1630</v>
+        <v>1628</v>
       </c>
       <c r="L384" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19833,10 +19831,10 @@
         <v>417</v>
       </c>
       <c r="C385" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E385" s="3" t="s">
-        <v>1631</v>
+        <v>1629</v>
       </c>
       <c r="F385" s="3" t="s">
         <v>966</v>
@@ -19848,7 +19846,7 @@
         <v>422</v>
       </c>
       <c r="J385" s="3" t="s">
-        <v>1632</v>
+        <v>1630</v>
       </c>
       <c r="L385" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19867,10 +19865,10 @@
         <v>424</v>
       </c>
       <c r="C386" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E386" s="3" t="s">
-        <v>1633</v>
+        <v>1631</v>
       </c>
       <c r="F386" s="3" t="s">
         <v>425</v>
@@ -19879,7 +19877,7 @@
         <v>969</v>
       </c>
       <c r="J386" s="3" t="s">
-        <v>1634</v>
+        <v>1632</v>
       </c>
       <c r="L386" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19898,22 +19896,22 @@
         <v>431</v>
       </c>
       <c r="C387" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E387" s="3" t="s">
-        <v>1635</v>
+        <v>1633</v>
       </c>
       <c r="F387" s="3" t="s">
         <v>434</v>
       </c>
       <c r="H387" s="3" t="s">
-        <v>1636</v>
+        <v>1634</v>
       </c>
       <c r="I387" s="3" t="s">
         <v>436</v>
       </c>
       <c r="J387" s="3" t="s">
-        <v>1637</v>
+        <v>1635</v>
       </c>
       <c r="L387" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19932,10 +19930,10 @@
         <v>438</v>
       </c>
       <c r="C388" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E388" s="3" t="s">
-        <v>1638</v>
+        <v>1636</v>
       </c>
       <c r="F388" s="3" t="s">
         <v>439</v>
@@ -19947,7 +19945,7 @@
         <v>442</v>
       </c>
       <c r="J388" s="3" t="s">
-        <v>1639</v>
+        <v>1637</v>
       </c>
       <c r="L388" s="3" t="str">
         <f t="shared" si="3"/>
@@ -19966,10 +19964,10 @@
         <v>444</v>
       </c>
       <c r="C389" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E389" s="3" t="s">
-        <v>1640</v>
+        <v>1638</v>
       </c>
       <c r="F389" s="3" t="s">
         <v>447</v>
@@ -19981,7 +19979,7 @@
         <v>449</v>
       </c>
       <c r="J389" s="3" t="s">
-        <v>1641</v>
+        <v>1639</v>
       </c>
       <c r="L389" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20000,13 +19998,13 @@
         <v>451</v>
       </c>
       <c r="C390" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E390" s="3" t="s">
-        <v>1642</v>
+        <v>1640</v>
       </c>
       <c r="F390" s="3" t="s">
-        <v>1643</v>
+        <v>1641</v>
       </c>
       <c r="H390" s="3" t="s">
         <v>1056</v>
@@ -20015,7 +20013,7 @@
         <v>454</v>
       </c>
       <c r="J390" s="3" t="s">
-        <v>1644</v>
+        <v>1642</v>
       </c>
       <c r="L390" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20034,22 +20032,22 @@
         <v>456</v>
       </c>
       <c r="C391" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E391" s="3" t="s">
-        <v>1645</v>
+        <v>1643</v>
       </c>
       <c r="F391" s="3" t="s">
-        <v>1646</v>
+        <v>1644</v>
       </c>
       <c r="H391" s="3" t="s">
         <v>1059</v>
       </c>
       <c r="I391" s="3" t="s">
-        <v>1647</v>
+        <v>1645</v>
       </c>
       <c r="J391" s="3" t="s">
-        <v>1648</v>
+        <v>1646</v>
       </c>
       <c r="L391" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20068,10 +20066,10 @@
         <v>461</v>
       </c>
       <c r="C392" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E392" s="3" t="s">
-        <v>1649</v>
+        <v>1647</v>
       </c>
       <c r="F392" s="3" t="s">
         <v>1061</v>
@@ -20080,10 +20078,10 @@
         <v>1063</v>
       </c>
       <c r="I392" s="3" t="s">
-        <v>1650</v>
+        <v>1648</v>
       </c>
       <c r="J392" s="3" t="s">
-        <v>1651</v>
+        <v>1649</v>
       </c>
       <c r="L392" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20102,10 +20100,10 @@
         <v>466</v>
       </c>
       <c r="C393" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E393" s="3" t="s">
-        <v>1652</v>
+        <v>1650</v>
       </c>
       <c r="F393" s="3" t="s">
         <v>1067</v>
@@ -20114,10 +20112,10 @@
         <v>1068</v>
       </c>
       <c r="I393" s="3" t="s">
-        <v>1653</v>
+        <v>1651</v>
       </c>
       <c r="J393" s="3" t="s">
-        <v>1654</v>
+        <v>1652</v>
       </c>
       <c r="L393" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20136,10 +20134,10 @@
         <v>470</v>
       </c>
       <c r="C394" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E394" s="3" t="s">
-        <v>1655</v>
+        <v>1653</v>
       </c>
       <c r="F394" s="3" t="s">
         <v>479</v>
@@ -20148,7 +20146,7 @@
         <v>1073</v>
       </c>
       <c r="J394" s="3" t="s">
-        <v>1656</v>
+        <v>1654</v>
       </c>
       <c r="L394" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20167,22 +20165,22 @@
         <v>484</v>
       </c>
       <c r="C395" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E395" s="3" t="s">
-        <v>1657</v>
+        <v>1655</v>
       </c>
       <c r="F395" s="3" t="s">
-        <v>1658</v>
+        <v>1656</v>
       </c>
       <c r="H395" s="3" t="s">
         <v>1086</v>
       </c>
       <c r="I395" s="3" t="s">
-        <v>1659</v>
+        <v>1657</v>
       </c>
       <c r="J395" s="3" t="s">
-        <v>1660</v>
+        <v>1658</v>
       </c>
       <c r="L395" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20201,10 +20199,10 @@
         <v>489</v>
       </c>
       <c r="C396" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E396" s="3" t="s">
-        <v>1661</v>
+        <v>1659</v>
       </c>
       <c r="F396" s="3" t="s">
         <v>1088</v>
@@ -20213,10 +20211,10 @@
         <v>1089</v>
       </c>
       <c r="I396" s="3" t="s">
-        <v>1662</v>
+        <v>1660</v>
       </c>
       <c r="J396" s="3" t="s">
-        <v>1663</v>
+        <v>1661</v>
       </c>
       <c r="L396" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20235,22 +20233,22 @@
         <v>494</v>
       </c>
       <c r="C397" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E397" s="3" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
       <c r="F397" s="3" t="s">
-        <v>1665</v>
+        <v>1663</v>
       </c>
       <c r="H397" s="3" t="s">
         <v>1093</v>
       </c>
       <c r="I397" s="3" t="s">
-        <v>1666</v>
+        <v>1664</v>
       </c>
       <c r="J397" s="3" t="s">
-        <v>1667</v>
+        <v>1665</v>
       </c>
       <c r="L397" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20269,13 +20267,13 @@
         <v>500</v>
       </c>
       <c r="C398" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E398" s="3" t="s">
-        <v>1668</v>
+        <v>1666</v>
       </c>
       <c r="F398" s="3" t="s">
-        <v>1458</v>
+        <v>1456</v>
       </c>
       <c r="H398" s="3" t="s">
         <v>1098</v>
@@ -20303,13 +20301,13 @@
         <v>508</v>
       </c>
       <c r="C399" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E399" s="3" t="s">
-        <v>1669</v>
+        <v>1667</v>
       </c>
       <c r="F399" s="3" t="s">
-        <v>1670</v>
+        <v>1668</v>
       </c>
       <c r="H399" s="3" t="s">
         <v>1101</v>
@@ -20318,7 +20316,7 @@
         <v>512</v>
       </c>
       <c r="J399" s="3" t="s">
-        <v>1671</v>
+        <v>1669</v>
       </c>
       <c r="L399" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20337,10 +20335,10 @@
         <v>514</v>
       </c>
       <c r="C400" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E400" s="3" t="s">
-        <v>1672</v>
+        <v>1670</v>
       </c>
       <c r="F400" s="3" t="s">
         <v>1105</v>
@@ -20349,10 +20347,10 @@
         <v>1106</v>
       </c>
       <c r="I400" s="3" t="s">
-        <v>1673</v>
+        <v>1671</v>
       </c>
       <c r="J400" s="3" t="s">
-        <v>1674</v>
+        <v>1672</v>
       </c>
       <c r="L400" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20371,10 +20369,10 @@
         <v>520</v>
       </c>
       <c r="C401" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E401" s="3" t="s">
-        <v>1675</v>
+        <v>1673</v>
       </c>
       <c r="F401" s="3" t="s">
         <v>523</v>
@@ -20383,10 +20381,10 @@
         <v>1116</v>
       </c>
       <c r="I401" s="3" t="s">
-        <v>1676</v>
+        <v>1674</v>
       </c>
       <c r="J401" s="3" t="s">
-        <v>1677</v>
+        <v>1675</v>
       </c>
       <c r="L401" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20405,10 +20403,10 @@
         <v>527</v>
       </c>
       <c r="C402" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E402" s="3" t="s">
-        <v>1678</v>
+        <v>1676</v>
       </c>
       <c r="F402" s="3" t="s">
         <v>530</v>
@@ -20420,7 +20418,7 @@
         <v>533</v>
       </c>
       <c r="J402" s="3" t="s">
-        <v>1679</v>
+        <v>1677</v>
       </c>
       <c r="L402" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20439,10 +20437,10 @@
         <v>535</v>
       </c>
       <c r="C403" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E403" s="3" t="s">
-        <v>1680</v>
+        <v>1678</v>
       </c>
       <c r="F403" s="3" t="s">
         <v>538</v>
@@ -20454,7 +20452,7 @@
         <v>540</v>
       </c>
       <c r="J403" s="3" t="s">
-        <v>1681</v>
+        <v>1679</v>
       </c>
       <c r="L403" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20473,25 +20471,25 @@
         <v>542</v>
       </c>
       <c r="C404" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E404" s="3" t="s">
-        <v>1682</v>
+        <v>1680</v>
       </c>
       <c r="F404" s="3" t="s">
         <v>545</v>
       </c>
       <c r="G404" s="3" t="s">
-        <v>1683</v>
+        <v>1681</v>
       </c>
       <c r="H404" s="3" t="s">
         <v>1127</v>
       </c>
       <c r="I404" s="3" t="s">
-        <v>1684</v>
+        <v>1682</v>
       </c>
       <c r="J404" s="3" t="s">
-        <v>1685</v>
+        <v>1683</v>
       </c>
       <c r="L404" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20510,22 +20508,22 @@
         <v>549</v>
       </c>
       <c r="C405" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E405" s="3" t="s">
-        <v>1686</v>
+        <v>1684</v>
       </c>
       <c r="F405" s="3" t="s">
-        <v>1687</v>
+        <v>1685</v>
       </c>
       <c r="H405" s="3" t="s">
         <v>1140</v>
       </c>
       <c r="I405" s="3" t="s">
-        <v>1688</v>
+        <v>1686</v>
       </c>
       <c r="J405" s="3" t="s">
-        <v>1689</v>
+        <v>1687</v>
       </c>
       <c r="L405" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20544,25 +20542,25 @@
         <v>555</v>
       </c>
       <c r="C406" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E406" s="3" t="s">
-        <v>1690</v>
+        <v>1688</v>
       </c>
       <c r="F406" s="3" t="s">
         <v>558</v>
       </c>
       <c r="G406" s="4" t="s">
-        <v>1691</v>
+        <v>1689</v>
       </c>
       <c r="H406" s="3" t="s">
         <v>1266</v>
       </c>
       <c r="I406" s="3" t="s">
-        <v>1692</v>
+        <v>1690</v>
       </c>
       <c r="J406" s="3" t="s">
-        <v>1693</v>
+        <v>1691</v>
       </c>
       <c r="L406" s="3" t="str">
         <f t="shared" si="3"/>
@@ -20581,19 +20579,19 @@
         <v>562</v>
       </c>
       <c r="C407" s="3" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="E407" s="3" t="s">
-        <v>1694</v>
+        <v>1692</v>
       </c>
       <c r="F407" s="3" t="s">
-        <v>1695</v>
+        <v>1693</v>
       </c>
       <c r="H407" s="3" t="s">
         <v>1298</v>
       </c>
       <c r="J407" s="3" t="s">
-        <v>1696</v>
+        <v>1694</v>
       </c>
       <c r="L407" s="3" t="str">
         <f t="shared" si="3"/>

</xml_diff>